<commit_message>
Improve scoreboard for portrait videos Improve score_tmpl
</commit_message>
<xml_diff>
--- a/in/score_tmpl.xlsx
+++ b/in/score_tmpl.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\vmshare\WORKSPACE\badminton_video_score\in\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1790F11F-EF02-4FDF-8E62-0E16F70FCF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03F00350-8883-4D68-8D83-B1BC42FD5F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21060" yWindow="180" windowWidth="7740" windowHeight="15300" xr2:uid="{925E6689-4E4F-41B8-BB79-50307361D580}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{925E6689-4E4F-41B8-BB79-50307361D580}"/>
   </bookViews>
   <sheets>
     <sheet name="scores" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Min</t>
   </si>
@@ -44,17 +44,20 @@
     <t>Trọng</t>
   </si>
   <si>
-    <t>Hảo</t>
+    <t>Cumulative score</t>
   </si>
   <si>
-    <t>Cumulative score</t>
+    <t>Sơn</t>
+  </si>
+  <si>
+    <t>Rally time</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="9"/>
       <color theme="1"/>
@@ -185,6 +188,13 @@
     <font>
       <sz val="9"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="0" tint="-0.249977111117893"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -531,11 +541,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -581,7 +593,38 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -911,32 +954,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A27867DC-DC27-4F1F-9822-9F44F2197CD4}">
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C2" s="1">
         <v>0</v>
@@ -952,8 +998,12 @@
         <f>D2</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G2" s="3">
+        <f>(A2*60+B2)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" t="str">
@@ -964,20 +1014,28 @@
         <f>IF(AND(D3="",E3=""),"",IF(LOWER(D3)="x", F2+1, F2))</f>
         <v/>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G3" s="3">
+        <f>(A3*60+B3)-(A2*60+B2)</f>
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" t="str">
-        <f t="shared" ref="E4:F62" si="0">IF(AND(C4="",D4=""),"",IF(LOWER(C4)="x", E3+1, E3))</f>
+        <f t="shared" ref="E4:F19" si="0">IF(AND(C4="",D4=""),"",IF(LOWER(C4)="x", E3+1, E3))</f>
         <v/>
       </c>
       <c r="F4" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G4" s="3">
+        <f t="shared" ref="G4:G62" si="1">(A4*60+B4)-(A3*60+B3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" t="str">
@@ -988,8 +1046,12 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G5" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" t="str">
@@ -1000,8 +1062,12 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G6" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" t="str">
@@ -1012,8 +1078,12 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G7" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" t="str">
@@ -1024,8 +1094,12 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G8" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" t="str">
@@ -1036,8 +1110,12 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G9" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" t="str">
@@ -1048,8 +1126,12 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G10" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" t="str">
@@ -1060,8 +1142,12 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G11" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" t="str">
@@ -1072,8 +1158,12 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G12" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" t="str">
@@ -1084,8 +1174,12 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G13" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" t="str">
@@ -1096,8 +1190,12 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G14" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" t="str">
@@ -1108,8 +1206,12 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G15" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" t="str">
@@ -1120,8 +1222,12 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="17" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="G16" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" t="str">
@@ -1132,8 +1238,12 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="18" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="G17" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" t="str">
@@ -1144,8 +1254,12 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="19" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="G18" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" t="str">
@@ -1156,528 +1270,714 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="20" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="G19" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E20:F35" si="2">IF(AND(C20="",D20=""),"",IF(LOWER(C20)="x", E19+1, E19))</f>
         <v/>
       </c>
       <c r="F20" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G20" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F21" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G21" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F22" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G22" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F23" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G23" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F24" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G24" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
       <c r="E25" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F25" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="26" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G25" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F26" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="27" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G26" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F27" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G27" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
       <c r="E28" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F28" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G28" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
       <c r="E29" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F29" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G29" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
       <c r="E30" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F30" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G30" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F31" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G31" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
       <c r="E32" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F32" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="33" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G32" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
       <c r="E33" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F33" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G33" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
       <c r="E34" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F34" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="35" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G34" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
       <c r="E35" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="F35" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="36" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G35" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E36:F51" si="3">IF(AND(C36="",D36=""),"",IF(LOWER(C36)="x", E35+1, E35))</f>
         <v/>
       </c>
       <c r="F36" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="37" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G36" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F37" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="38" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G37" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F38" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G38" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C39" s="1"/>
       <c r="D39" s="1"/>
       <c r="E39" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F39" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="40" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G39" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
       <c r="E40" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F40" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="41" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G40" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C41" s="1"/>
       <c r="D41" s="1"/>
       <c r="E41" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F41" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="42" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G41" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
       <c r="E42" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F42" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="43" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G42" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
       <c r="E43" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F43" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="44" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G43" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
       <c r="E44" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F44" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="45" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G44" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C45" s="1"/>
       <c r="D45" s="1"/>
       <c r="E45" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F45" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="46" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G45" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
       <c r="E46" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F46" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="47" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G46" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C47" s="1"/>
       <c r="D47" s="1"/>
       <c r="E47" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F47" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="48" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G47" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C48" s="1"/>
       <c r="D48" s="1"/>
       <c r="E48" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F48" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="49" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G48" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C49" s="1"/>
       <c r="D49" s="1"/>
       <c r="E49" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F49" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="50" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G49" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C50" s="1"/>
       <c r="D50" s="1"/>
       <c r="E50" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F50" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="51" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G50" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C51" s="1"/>
       <c r="D51" s="1"/>
       <c r="E51" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="F51" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="52" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G51" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C52" s="1"/>
       <c r="D52" s="1"/>
       <c r="E52" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E52:F62" si="4">IF(AND(C52="",D52=""),"",IF(LOWER(C52)="x", E51+1, E51))</f>
         <v/>
       </c>
       <c r="F52" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="53" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G52" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C53" s="1"/>
       <c r="D53" s="1"/>
       <c r="E53" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F53" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="54" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G53" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C54" s="1"/>
       <c r="D54" s="1"/>
       <c r="E54" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F54" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="55" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G54" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C55" s="1"/>
       <c r="D55" s="1"/>
       <c r="E55" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F55" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="56" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G55" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C56" s="1"/>
       <c r="D56" s="1"/>
       <c r="E56" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F56" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="57" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G56" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C57" s="1"/>
       <c r="D57" s="1"/>
       <c r="E57" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F57" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="58" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G57" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C58" s="1"/>
       <c r="D58" s="1"/>
       <c r="E58" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F58" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="59" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G58" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C59" s="1"/>
       <c r="D59" s="1"/>
       <c r="E59" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F59" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="60" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G59" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C60" s="1"/>
       <c r="D60" s="1"/>
       <c r="E60" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F60" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="61" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G60" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
       <c r="E61" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F61" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="62" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G61" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C62" s="1"/>
       <c r="D62" s="1"/>
       <c r="E62" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="F62" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="63" spans="3:6" x14ac:dyDescent="0.2">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G62" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C63" s="1"/>
       <c r="D63" s="1"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="G2:G62">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
+      <formula>25</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G61">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>